<commit_message>
Get base pop freqs
</commit_message>
<xml_diff>
--- a/Raw_data/RIL_IDs_FF_Hamlin_etal_2025.xlsx
+++ b/Raw_data/RIL_IDs_FF_Hamlin_etal_2025.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailmissouri-my.sharepoint.com/personal/svqht_umsystem_edu/Documents/Flying Flies Phenotyping/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kingeg/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C441A8BD-356A-1641-BF62-FED9F1301B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{222873FC-CCF5-2B4F-8565-2FC6785C04E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4360" yWindow="2260" windowWidth="28040" windowHeight="17180" xr2:uid="{7FE76E8B-8C70-514D-AFDA-E9AAA365A388}"/>
   </bookViews>
   <sheets>
     <sheet name="RIL_IDs" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,6 +36,14 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+  <si>
+    <t>ril</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -412,327 +420,480 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F729CA82-AF87-9642-981D-C4A22E878C4E}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A1" s="1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>11004</v>
       </c>
-      <c r="B1" s="1">
-        <v>11009</v>
-      </c>
-      <c r="C1" s="1">
-        <v>11012</v>
-      </c>
-      <c r="D1" s="1">
-        <v>11016</v>
-      </c>
-      <c r="E1" s="1">
-        <v>11037</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+    </row>
+    <row r="3" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
         <v>11038</v>
       </c>
-      <c r="B2" s="1">
-        <v>11044</v>
-      </c>
-      <c r="C2" s="1">
-        <v>11052</v>
-      </c>
-      <c r="D2" s="1">
-        <v>11062</v>
-      </c>
-      <c r="E2" s="1">
-        <v>11074</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+    </row>
+    <row r="4" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
         <v>11110</v>
       </c>
-      <c r="B3" s="1">
-        <v>11117</v>
-      </c>
-      <c r="C3" s="1">
-        <v>11122</v>
-      </c>
-      <c r="D3" s="1">
-        <v>11149</v>
-      </c>
-      <c r="E3" s="1">
-        <v>11153</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
+    </row>
+    <row r="5" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <v>11155</v>
       </c>
-      <c r="B4" s="1">
-        <v>11159</v>
-      </c>
-      <c r="C4" s="1">
-        <v>11162</v>
-      </c>
-      <c r="D4" s="1">
-        <v>11185</v>
-      </c>
-      <c r="E4" s="1">
-        <v>11192</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+    </row>
+    <row r="6" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
         <v>11196</v>
       </c>
-      <c r="B5" s="1">
-        <v>11216</v>
-      </c>
-      <c r="C5" s="1">
-        <v>11228</v>
-      </c>
-      <c r="D5" s="1">
-        <v>11232</v>
-      </c>
-      <c r="E5" s="1">
-        <v>11239</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+    </row>
+    <row r="7" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
         <v>11255</v>
       </c>
-      <c r="B6" s="1">
-        <v>11265</v>
-      </c>
-      <c r="C6" s="1">
-        <v>11298</v>
-      </c>
-      <c r="D6" s="1">
-        <v>11299</v>
-      </c>
-      <c r="E6" s="1">
-        <v>11300</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+    </row>
+    <row r="8" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
         <v>11303</v>
       </c>
-      <c r="B7" s="1">
-        <v>11305</v>
-      </c>
-      <c r="C7" s="1">
-        <v>11310</v>
-      </c>
-      <c r="D7" s="1">
-        <v>11316</v>
-      </c>
-      <c r="E7" s="1">
-        <v>11321</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
+    </row>
+    <row r="9" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
         <v>11328</v>
       </c>
-      <c r="B8" s="1">
-        <v>11355</v>
-      </c>
-      <c r="C8" s="1">
-        <v>11358</v>
-      </c>
-      <c r="D8" s="1">
-        <v>11360</v>
-      </c>
-      <c r="E8" s="1">
-        <v>11361</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
+    </row>
+    <row r="10" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
         <v>11369</v>
       </c>
-      <c r="B9" s="1">
-        <v>11374</v>
-      </c>
-      <c r="C9" s="1">
-        <v>11375</v>
-      </c>
-      <c r="D9" s="1">
-        <v>11376</v>
-      </c>
-      <c r="E9" s="1">
-        <v>11381</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
+    </row>
+    <row r="11" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
         <v>11410</v>
       </c>
-      <c r="B10" s="1">
-        <v>11416</v>
-      </c>
-      <c r="C10" s="1">
-        <v>11420</v>
-      </c>
-      <c r="D10" s="1">
-        <v>11464</v>
-      </c>
-      <c r="E10" s="1">
-        <v>11465</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
+    </row>
+    <row r="12" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
         <v>11466</v>
       </c>
-      <c r="B11" s="1">
-        <v>11481</v>
-      </c>
-      <c r="C11" s="1">
-        <v>12002</v>
-      </c>
-      <c r="D11" s="1">
-        <v>12010</v>
-      </c>
-      <c r="E11" s="1">
-        <v>12014</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+    </row>
+    <row r="13" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
         <v>12021</v>
       </c>
-      <c r="B12" s="1">
-        <v>12022</v>
-      </c>
-      <c r="C12" s="1">
-        <v>12028</v>
-      </c>
-      <c r="D12" s="1">
-        <v>12039</v>
-      </c>
-      <c r="E12" s="1">
-        <v>12043</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
+    </row>
+    <row r="14" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
         <v>12050</v>
       </c>
-      <c r="B13" s="1">
-        <v>12075</v>
-      </c>
-      <c r="C13" s="1">
-        <v>12080</v>
-      </c>
-      <c r="D13" s="1">
-        <v>12097</v>
-      </c>
-      <c r="E13" s="1">
-        <v>12114</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
+    </row>
+    <row r="15" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
         <v>12123</v>
       </c>
-      <c r="B14" s="1">
-        <v>12130</v>
-      </c>
-      <c r="C14" s="1">
-        <v>12138</v>
-      </c>
-      <c r="D14" s="1">
-        <v>12145</v>
-      </c>
-      <c r="E14" s="1">
-        <v>12159</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+    </row>
+    <row r="16" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
         <v>12169</v>
-      </c>
-      <c r="B15" s="1">
-        <v>12190</v>
-      </c>
-      <c r="C15" s="1">
-        <v>12191</v>
-      </c>
-      <c r="D15" s="1">
-        <v>12234</v>
-      </c>
-      <c r="E15" s="1">
-        <v>12243</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="22" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <v>12253</v>
-      </c>
-      <c r="B16" s="1">
-        <v>12258</v>
-      </c>
-      <c r="C16" s="1">
-        <v>12270</v>
-      </c>
-      <c r="D16" s="1">
-        <v>12272</v>
-      </c>
-      <c r="E16" s="1">
-        <v>12278</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="22" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>12279</v>
-      </c>
-      <c r="B17" s="1">
-        <v>12285</v>
-      </c>
-      <c r="C17" s="1">
-        <v>12300</v>
-      </c>
-      <c r="D17" s="1">
-        <v>12301</v>
-      </c>
-      <c r="E17" s="1">
-        <v>12304</v>
+        <v>12253</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="22" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>12316</v>
-      </c>
-      <c r="B18" s="1">
-        <v>12333</v>
-      </c>
-      <c r="C18" s="1">
-        <v>12348</v>
-      </c>
-      <c r="D18" s="1">
-        <v>12357</v>
-      </c>
-      <c r="E18" s="1">
-        <v>12363</v>
+        <v>12279</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="22" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>12372</v>
-      </c>
-      <c r="B19" s="1">
-        <v>12381</v>
-      </c>
-      <c r="C19" s="1">
-        <v>12390</v>
+        <v>12316</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>12372</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>11009</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>11044</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>11117</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>11159</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>11216</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>11265</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>11305</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>11355</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>11374</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>11416</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>11481</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="22" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>12022</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>12075</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>12130</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>12190</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>12258</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>12285</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>12333</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>12381</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>11012</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>11052</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>11122</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>11162</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>11228</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>11298</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>11310</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>11358</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>11375</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>11420</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>12002</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>12028</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>12080</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>12138</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>12191</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>12270</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>12300</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>12348</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>12390</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>11016</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>11062</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>11149</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>11185</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>11232</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>11299</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>11316</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>11360</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>11376</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>11464</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>12010</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>12039</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>12097</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>12145</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>12234</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>12272</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>12301</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>12357</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>11037</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>11074</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>11153</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>11192</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>11239</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>11300</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>11321</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>11361</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>11381</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>11465</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>12014</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>12043</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>12114</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>12159</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>12243</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>12278</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>12304</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" ht="22" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
+        <v>12363</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>